<commit_message>
chore: update CA template
</commit_message>
<xml_diff>
--- a/next/app/zev-unit-activities/lib/credit-applications/templates/credit_application_supplier_template.xlsx
+++ b/next/app/zev-unit-activities/lib/credit-applications/templates/credit_application_supplier_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timchen/Desktop/zeva/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8076AD1-C586-A140-8654-293609F10DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9A08DD-F683-394E-8DEA-1F628BD170ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5620" yWindow="2760" windowWidth="27240" windowHeight="16440" xr2:uid="{515AB8EB-AA8F-2C43-9A6B-8AF89862BE7B}"/>
+    <workbookView xWindow="10640" yWindow="2740" windowWidth="27240" windowHeight="16440" xr2:uid="{515AB8EB-AA8F-2C43-9A6B-8AF89862BE7B}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Make</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>(1) If a row is not empty, then no cell within that row may be empty.</t>
+  </si>
+  <si>
+    <t>(6) Ensure there are no leading or trailing spaces</t>
+  </si>
+  <si>
+    <t>(7) Do not enter any dates later than the submission date of this application</t>
   </si>
 </sst>
 </file>
@@ -472,10 +478,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC198ED0-26FB-CD41-B8E5-195ADA9EB37D}">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="60.33203125" customWidth="1"/>
+    <col min="1" max="1" width="73.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -536,6 +542,16 @@
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CA template (#550)
</commit_message>
<xml_diff>
--- a/next/app/zev-unit-activities/lib/credit-applications/templates/credit_application_supplier_template.xlsx
+++ b/next/app/zev-unit-activities/lib/credit-applications/templates/credit_application_supplier_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timchen/Desktop/zeva/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8076AD1-C586-A140-8654-293609F10DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9A08DD-F683-394E-8DEA-1F628BD170ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5620" yWindow="2760" windowWidth="27240" windowHeight="16440" xr2:uid="{515AB8EB-AA8F-2C43-9A6B-8AF89862BE7B}"/>
+    <workbookView xWindow="10640" yWindow="2740" windowWidth="27240" windowHeight="16440" xr2:uid="{515AB8EB-AA8F-2C43-9A6B-8AF89862BE7B}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Make</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>(1) If a row is not empty, then no cell within that row may be empty.</t>
+  </si>
+  <si>
+    <t>(6) Ensure there are no leading or trailing spaces</t>
+  </si>
+  <si>
+    <t>(7) Do not enter any dates later than the submission date of this application</t>
   </si>
 </sst>
 </file>
@@ -472,10 +478,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC198ED0-26FB-CD41-B8E5-195ADA9EB37D}">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="60.33203125" customWidth="1"/>
+    <col min="1" max="1" width="73.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -536,6 +542,16 @@
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>